<commit_message>
Update Remap Draft for Sanhua
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/SanhuaRemapDraft.xlsx
+++ b/Data/RemapDrafts/SanhuaRemapDraft.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexX\Documents\Games\Mods\Repos\Anime-Game-Remap\Data\RemapDrafts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A467BCF-F9B1-4F12-8CE5-911DCC24BC7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96F85D45-C778-4015-B577-407FBD54A7A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{AFEAC171-B6A1-42D5-A35D-F87A53EF5600}"/>
   </bookViews>
   <sheets>
-    <sheet name="2.4 -Sanhua to SanhuaExorcist" sheetId="1" r:id="rId1"/>
+    <sheet name="2.5 -Sanhua to SanhuaExorcist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2.4 -Sanhua to SanhuaExorcist'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2.5 -Sanhua to SanhuaExorcist'!$A$1:$D$209</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="66">
   <si>
     <t>Uncertainty</t>
   </si>
@@ -49,6 +49,192 @@
   </si>
   <si>
     <t>SanhuaExorcist</t>
+  </si>
+  <si>
+    <t>right shoulder</t>
+  </si>
+  <si>
+    <t>left shoulder</t>
+  </si>
+  <si>
+    <t>left palm</t>
+  </si>
+  <si>
+    <t>left wrist</t>
+  </si>
+  <si>
+    <t>right palm</t>
+  </si>
+  <si>
+    <t>left lower arm, upper part</t>
+  </si>
+  <si>
+    <t>left upper arm, upper part</t>
+  </si>
+  <si>
+    <t>right wrist</t>
+  </si>
+  <si>
+    <t>right lower arm, upper part</t>
+  </si>
+  <si>
+    <t>right upper arm, upper part</t>
+  </si>
+  <si>
+    <t>Bow behind Sanhua's head</t>
+  </si>
+  <si>
+    <t>chest</t>
+  </si>
+  <si>
+    <t>dangling string from Sanhua's right chest</t>
+  </si>
+  <si>
+    <t>right, top string knot tied to Sanhua's right neck</t>
+  </si>
+  <si>
+    <t>right earing</t>
+  </si>
+  <si>
+    <t>dangling string from Sanhua's right beret</t>
+  </si>
+  <si>
+    <t>left, top string knot tied to Sanhua's right neck</t>
+  </si>
+  <si>
+    <t>left, top dangling thing from Sanhua's back skirt</t>
+  </si>
+  <si>
+    <t>right, top dangling thing from Sanhua's back skirt</t>
+  </si>
+  <si>
+    <t>left calf</t>
+  </si>
+  <si>
+    <t>left thigh, upper part</t>
+  </si>
+  <si>
+    <t>left ankle, upper part</t>
+  </si>
+  <si>
+    <t>left thigh gap, lower part</t>
+  </si>
+  <si>
+    <t>right thigh, lower part</t>
+  </si>
+  <si>
+    <t>left thigh, lower part</t>
+  </si>
+  <si>
+    <t>right calf</t>
+  </si>
+  <si>
+    <t>right ankle, upper part</t>
+  </si>
+  <si>
+    <t>Sanhua's right waist underneath skirt</t>
+  </si>
+  <si>
+    <t>Sanhua's skirt front, right upper part</t>
+  </si>
+  <si>
+    <t>Sanhua's skirt front upper part</t>
+  </si>
+  <si>
+    <t>Sanhua's skirt front, left upper part</t>
+  </si>
+  <si>
+    <t>Sanhua's skirt back upper part</t>
+  </si>
+  <si>
+    <t>Sanhua's back skirt, middle part</t>
+  </si>
+  <si>
+    <t>Sanhua's skirt, bottom part 2</t>
+  </si>
+  <si>
+    <t>Sanhua's dangling belt at left front bottom skirt</t>
+  </si>
+  <si>
+    <t>Sanhua's dangling charm from front right waist</t>
+  </si>
+  <si>
+    <t>Sanhua's skirt front middle part</t>
+  </si>
+  <si>
+    <t>Sanhua's right top, dangling belt from her back skirt</t>
+  </si>
+  <si>
+    <t>Sanhua's left top, dangling belt from her back skirt</t>
+  </si>
+  <si>
+    <t>Sanhua's belt at right front top skirt</t>
+  </si>
+  <si>
+    <t>Sanhua's back skirt, upper part 2</t>
+  </si>
+  <si>
+    <t>Sanhua's left back skirt, upper part 2</t>
+  </si>
+  <si>
+    <t>Sanhua's right back skirt, upper part 2</t>
+  </si>
+  <si>
+    <t>Sanhua's back skirt, middle part 2</t>
+  </si>
+  <si>
+    <t>Sanhua's left back skirt, middle part</t>
+  </si>
+  <si>
+    <t>Sanhua's left back skirt, midde part 2</t>
+  </si>
+  <si>
+    <t>Sanhua's left back skirt, bottom part 2</t>
+  </si>
+  <si>
+    <t>Sanhua's left back skirt, middle part 3</t>
+  </si>
+  <si>
+    <t>Sanhua's back skirt, bottom part</t>
+  </si>
+  <si>
+    <t>Sanhua's left foot</t>
+  </si>
+  <si>
+    <t>Sanhua's left toes</t>
+  </si>
+  <si>
+    <t>Sanhua's right foot</t>
+  </si>
+  <si>
+    <t>left bottom, dangling thing from Sanhua's back skirt</t>
+  </si>
+  <si>
+    <t>Sanhua's skirt, front bottom right part</t>
+  </si>
+  <si>
+    <t>Sanhua's back skirt, middle part 3</t>
+  </si>
+  <si>
+    <t>Sanhua's back skirt,middle part 2</t>
+  </si>
+  <si>
+    <t>Sanhua's back skirt, bottom part 2</t>
+  </si>
+  <si>
+    <t>Sanhua's right skirt, middle part 3</t>
+  </si>
+  <si>
+    <t>Sanhua's right skirt, middle part 2</t>
+  </si>
+  <si>
+    <t>Sanhua's right skirt, bottom part</t>
+  </si>
+  <si>
+    <t>Sanhua's right toes</t>
+  </si>
+  <si>
+    <t>right bottom, dangling thing from Sanhua's back skirt</t>
   </si>
 </sst>
 </file>
@@ -99,7 +285,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -447,1047 +643,1865 @@
       <c r="A2">
         <v>0</v>
       </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
+      <c r="B9">
+        <v>17</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
+      <c r="B10">
+        <v>8</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
+      <c r="B11">
+        <v>9</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
+      <c r="B12">
+        <v>10</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
+      <c r="B13">
+        <v>7</v>
+      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
+      <c r="B14">
+        <v>11</v>
+      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
+      <c r="B15">
+        <v>12</v>
+      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B16">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B17">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>17</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>18</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B22">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>22</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B24">
+        <v>24</v>
+      </c>
+      <c r="D24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>25</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B27">
+        <v>146</v>
+      </c>
+      <c r="C27">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>26</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B28">
+        <v>68</v>
+      </c>
+      <c r="C28">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>27</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B29">
+        <v>38</v>
+      </c>
+      <c r="D29" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>28</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B30">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>30</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B32">
+        <v>22</v>
+      </c>
+      <c r="D32" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>31</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B33">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>33</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B35">
+        <v>91</v>
+      </c>
+      <c r="D35" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>34</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B36">
+        <v>32</v>
+      </c>
+      <c r="D36" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>35</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B37">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>36</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B38">
+        <v>27</v>
+      </c>
+      <c r="D38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>37</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B39">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>38</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B40">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>39</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B41">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>40</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B42">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>41</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B43">
+        <v>25</v>
+      </c>
+      <c r="D43" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>42</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B44">
+        <v>107</v>
+      </c>
+      <c r="D44" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>43</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B45">
+        <v>42</v>
+      </c>
+      <c r="D45" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>44</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B46">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>45</v>
       </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B47">
+        <v>34</v>
+      </c>
+      <c r="D47" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>46</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B48">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>47</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B49">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>48</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B50">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>49</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B51">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>50</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B52">
+        <v>36</v>
+      </c>
+      <c r="D52" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>51</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>52</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>53</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>54</v>
       </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B56">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>55</v>
       </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B57">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>56</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>57</v>
       </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59">
+        <v>0.2</v>
+      </c>
+      <c r="D59" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>59</v>
       </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>60</v>
       </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B62">
+        <v>24</v>
+      </c>
+      <c r="C62">
+        <v>0.2</v>
+      </c>
+      <c r="D62" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>61</v>
       </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B63">
+        <v>24</v>
+      </c>
+      <c r="C63">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>62</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B64">
+        <v>52</v>
+      </c>
+      <c r="C64">
+        <v>0.2</v>
+      </c>
+      <c r="D64" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>63</v>
       </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B65">
+        <v>1</v>
+      </c>
+      <c r="D65" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>64</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>65</v>
       </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67">
+        <v>0.2</v>
+      </c>
+      <c r="D67" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>66</v>
       </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B68">
+        <v>1</v>
+      </c>
+      <c r="C68">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>67</v>
       </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>68</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>69</v>
       </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B71">
+        <v>49</v>
+      </c>
+      <c r="D71" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>70</v>
       </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B72">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>71</v>
       </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B73">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>72</v>
       </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B74">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>73</v>
       </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B75">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>74</v>
       </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B76">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>75</v>
       </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B77">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>76</v>
       </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B78">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>77</v>
       </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B79">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>78</v>
       </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B80">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>79</v>
       </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B81">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>80</v>
       </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B82">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>81</v>
       </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B83">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>82</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>83</v>
       </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B85">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>84</v>
       </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B86">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>85</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>86</v>
       </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B88">
+        <v>152</v>
+      </c>
+      <c r="D88" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>87</v>
       </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B89">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>88</v>
       </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B90">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>89</v>
       </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B91">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>90</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>91</v>
       </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B93">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>92</v>
       </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B94">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>93</v>
       </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B95">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>94</v>
       </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B96">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>95</v>
       </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B97">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>96</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>97</v>
       </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B99">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>98</v>
       </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B100">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>99</v>
       </c>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B101">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>100</v>
       </c>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B102">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>101</v>
       </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B103">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>102</v>
       </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B104">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>103</v>
       </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B105">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>104</v>
       </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B106">
+        <v>157</v>
+      </c>
+      <c r="D106" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>105</v>
       </c>
-    </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B107">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>106</v>
       </c>
-    </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B108">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>107</v>
       </c>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B109">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>108</v>
       </c>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>109</v>
       </c>
-    </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B111">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>110</v>
       </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B112">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>111</v>
       </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B113">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>112</v>
       </c>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>113</v>
       </c>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>114</v>
       </c>
-    </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B116">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>115</v>
       </c>
-    </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B117">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>116</v>
       </c>
-    </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B118">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>117</v>
       </c>
-    </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B119">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>118</v>
       </c>
-    </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B120">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>119</v>
       </c>
-    </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B121">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>120</v>
       </c>
-    </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B122">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>121</v>
       </c>
-    </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B123">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>122</v>
       </c>
-    </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B124">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>123</v>
       </c>
-    </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B125">
+        <v>81</v>
+      </c>
+      <c r="D125" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>124</v>
       </c>
-    </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B126">
+        <v>83</v>
+      </c>
+      <c r="D126" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>125</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>126</v>
       </c>
-    </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B128">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>127</v>
       </c>
-    </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B129">
+        <v>71</v>
+      </c>
+      <c r="D129" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>128</v>
       </c>
-    </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B130">
+        <v>85</v>
+      </c>
+      <c r="D130" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>129</v>
       </c>
-    </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B131">
+        <v>63</v>
+      </c>
+      <c r="D131" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>130</v>
       </c>
-    </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B132">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>131</v>
       </c>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>132</v>
       </c>
-    </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B134">
+        <v>86</v>
+      </c>
+      <c r="D134" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>133</v>
       </c>
-    </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B135">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>134</v>
       </c>
-    </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B136">
+        <v>88</v>
+      </c>
+      <c r="D136" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>135</v>
       </c>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>136</v>
       </c>
-    </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B138">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>137</v>
       </c>
-    </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B139">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>138</v>
       </c>
-    </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B140">
+        <v>90</v>
+      </c>
+      <c r="D140" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>139</v>
       </c>
-    </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B141">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>140</v>
       </c>
-    </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B142">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>141</v>
       </c>
-    </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B143">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>142</v>
       </c>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>143</v>
       </c>
     </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>144</v>
       </c>
-    </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B146">
+        <v>77</v>
+      </c>
+      <c r="D146" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>145</v>
       </c>
-    </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B147">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>146</v>
       </c>
-    </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B148">
+        <v>79</v>
+      </c>
+      <c r="C148">
+        <v>0.1</v>
+      </c>
+      <c r="D148" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>147</v>
       </c>
-    </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B149">
+        <v>80</v>
+      </c>
+      <c r="C149">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>148</v>
       </c>
-    </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B150">
+        <v>72</v>
+      </c>
+      <c r="D150" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>149</v>
       </c>
-    </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B151">
+        <v>73</v>
+      </c>
+      <c r="C151">
+        <v>0.1</v>
+      </c>
+      <c r="D151" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>150</v>
       </c>
-    </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B152">
+        <v>74</v>
+      </c>
+      <c r="C152">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>151</v>
       </c>
-    </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B153">
+        <v>75</v>
+      </c>
+      <c r="C153">
+        <v>0.2</v>
+      </c>
+      <c r="D153" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>152</v>
       </c>
-    </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B154">
+        <v>147</v>
+      </c>
+      <c r="C154">
+        <v>0.2</v>
+      </c>
+      <c r="D154" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>153</v>
       </c>
-    </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B155">
+        <v>133</v>
+      </c>
+      <c r="C155">
+        <v>0.3</v>
+      </c>
+      <c r="D155" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>154</v>
       </c>
-    </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B156">
+        <v>148</v>
+      </c>
+      <c r="C156">
+        <v>0.2</v>
+      </c>
+      <c r="D156" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>155</v>
       </c>
-    </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B157">
+        <v>182</v>
+      </c>
+      <c r="C157">
+        <v>0.2</v>
+      </c>
+      <c r="D157" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>156</v>
       </c>
-    </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B158">
+        <v>131</v>
+      </c>
+      <c r="C158">
+        <v>0.2</v>
+      </c>
+      <c r="D158" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>157</v>
       </c>
-    </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B159">
+        <v>164</v>
+      </c>
+      <c r="C159">
+        <v>0.4</v>
+      </c>
+      <c r="D159" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>158</v>
       </c>
-    </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B160">
+        <v>142</v>
+      </c>
+      <c r="D160" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>159</v>
       </c>
-    </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B161">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>160</v>
       </c>
-    </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B162">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>161</v>
       </c>
-    </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B163">
+        <v>169</v>
+      </c>
+      <c r="C163">
+        <v>0.2</v>
+      </c>
+      <c r="D163" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>162</v>
       </c>
-    </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B164">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>163</v>
       </c>
-    </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B165">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>164</v>
       </c>
-    </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B166">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>165</v>
       </c>
-    </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B167">
+        <v>176</v>
+      </c>
+      <c r="C167">
+        <v>0.2</v>
+      </c>
+      <c r="D167" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>166</v>
       </c>
-    </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B168">
+        <v>177</v>
+      </c>
+      <c r="C168">
+        <v>0.2</v>
+      </c>
+      <c r="D168" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>167</v>
       </c>
-    </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B169">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>168</v>
       </c>
-    </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B170">
+        <v>73</v>
+      </c>
+      <c r="C170">
+        <v>0.2</v>
+      </c>
+      <c r="D170" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>169</v>
       </c>
-    </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B171">
+        <v>162</v>
+      </c>
+      <c r="C171">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>170</v>
       </c>
-    </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B172">
+        <v>164</v>
+      </c>
+      <c r="C172">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>171</v>
       </c>
-    </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B173">
+        <v>164</v>
+      </c>
+      <c r="C173">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>172</v>
       </c>
-    </row>
-    <row r="175" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B174">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>173</v>
       </c>
-    </row>
-    <row r="176" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B175">
+        <v>137</v>
+      </c>
+      <c r="D175" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>174</v>
       </c>
-    </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B176">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>175</v>
       </c>
-    </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B177">
+        <v>132</v>
+      </c>
+      <c r="D177" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>176</v>
       </c>
-    </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B178">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>177</v>
       </c>
-    </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B179">
+        <v>172</v>
+      </c>
+      <c r="D179" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>178</v>
       </c>
-    </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B180">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>179</v>
       </c>
-    </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B181">
+        <v>149</v>
+      </c>
+      <c r="D181" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>180</v>
       </c>
-    </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B182">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>181</v>
       </c>
-    </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B183">
+        <v>186</v>
+      </c>
+      <c r="D183" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>182</v>
       </c>
-    </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B184">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>183</v>
       </c>
-    </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B185">
+        <v>189</v>
+      </c>
+      <c r="D185" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>184</v>
       </c>
-    </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B186">
+        <v>184</v>
+      </c>
+      <c r="D186" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>185</v>
       </c>
-    </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B187">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>186</v>
       </c>
-    </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B188">
+        <v>125</v>
+      </c>
+      <c r="D188" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>187</v>
       </c>
-    </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B189">
+        <v>126</v>
+      </c>
+      <c r="D189" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>188</v>
       </c>
-    </row>
-    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B190">
+        <v>123</v>
+      </c>
+      <c r="D190" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>189</v>
       </c>
-    </row>
-    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B191">
+        <v>155</v>
+      </c>
+      <c r="D191" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>190</v>
       </c>
-    </row>
-    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B192">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>191</v>
       </c>
-    </row>
-    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B193">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>192</v>
       </c>
     </row>
-    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>193</v>
       </c>
-    </row>
-    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B195">
+        <v>161</v>
+      </c>
+      <c r="D195" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>194</v>
       </c>
-    </row>
-    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B196">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>195</v>
       </c>
-    </row>
-    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B197">
+        <v>175</v>
+      </c>
+      <c r="D197" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>196</v>
       </c>
-    </row>
-    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B198">
+        <v>150</v>
+      </c>
+      <c r="D198" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>197</v>
       </c>
-    </row>
-    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B199">
+        <v>181</v>
+      </c>
+      <c r="D199" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>198</v>
       </c>
-    </row>
-    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B200">
+        <v>178</v>
+      </c>
+      <c r="D200" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>199</v>
       </c>
-    </row>
-    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B201">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>200</v>
       </c>
-    </row>
-    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B202">
+        <v>174</v>
+      </c>
+      <c r="D202" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>201</v>
       </c>
-    </row>
-    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B203">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>202</v>
       </c>
-    </row>
-    <row r="205" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B204">
+        <v>180</v>
+      </c>
+      <c r="D204" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>203</v>
       </c>
-    </row>
-    <row r="206" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B205">
+        <v>124</v>
+      </c>
+      <c r="D205" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>204</v>
       </c>
     </row>
-    <row r="207" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>205</v>
       </c>
-    </row>
-    <row r="208" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B207">
+        <v>159</v>
+      </c>
+      <c r="D207" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>206</v>
       </c>
-    </row>
-    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B208">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>207</v>
       </c>
+      <c r="B209">
+        <v>160</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1" xr:uid="{26373B65-F8B3-4A4D-95F8-AB47F03B2133}"/>
+  <autoFilter ref="A1:D209" xr:uid="{26373B65-F8B3-4A4D-95F8-AB47F03B2133}"/>
   <conditionalFormatting sqref="B2:B209">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>